<commit_message>
Door Access/Integrations 상품 매핑 추가 및 NocoDB 타임스탬프 KST 변환 지원
Door Access 31개 + Integrations 6개 신규 등록 상품을 sync_naver_ids_to_nocodb.py의
TARGET_PRODUCTS에 반영하고, 그 등록 결과(registered_log.json)와 갱신된 엑셀
템플릿을 함께 기록. nocodb_client.py에는 NocoDB가 UTC로 저장하는 CreatedAt/
UpdatedAt을 KST로 자동 변환해 돌려주는 로직을 추가해, 대시보드에서 타임스탬프가
항상 한국 시간 기준으로 보이게 함. 이전 세션에서 작업했지만 커밋되지 않았던
변경사항을 정리해 반영.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/naver_상품등록_템플릿.xlsx
+++ b/naver_상품등록_템플릿.xlsx
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3633,6 +3633,1751 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>UniFi Reader Junction Box</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>UniFi Reader Junction Box</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E88" t="n">
+        <v>66200</v>
+      </c>
+      <c r="F88" t="n">
+        <v>60200</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>UniFi Reader Junction Box</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>reader-junction-box</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>5</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer Table Stand</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer Table Stand</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E89" t="n">
+        <v>60800</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer Table Stand</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>intercom-viewer-table-stand</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>5</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>UniFi Gate Hub</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>UniFi Gate Hub</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E90" t="n">
+        <v>624900</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>UniFi Gate Hub</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>gate-hub</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>5</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Flush Mount</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Flush Mount</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E91" t="n">
+        <v>99000</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Flush Mount</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>intercom-flush-mount</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>5</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>UniFi Junction Utility</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>UniFi Junction Utility</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E92" t="n">
+        <v>219700</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>UniFi Junction Utility</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>junction-utility</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>5</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>UniFi Magnetic Lock</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>UniFi Magnetic Lock</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E93" t="n">
+        <v>271500</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>UniFi Magnetic Lock</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>magnetic-lock</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>5</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>UniFi Gate Starter Kit</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>UniFi Gate Starter Kit</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1433700</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>UniFi Gate Starter Kit</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>gate-starter-kit</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>5</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub Mini</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub Mini</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E95" t="n">
+        <v>250700</v>
+      </c>
+      <c r="F95" t="n">
+        <v>212200</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub Mini</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>door-hub-mini</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>5</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E96" t="n">
+        <v>354400</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Viewer</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>intercom-viewer</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>5</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Surface Angle Mount</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Surface Angle Mount</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E97" t="n">
+        <v>95700</v>
+      </c>
+      <c r="F97" t="n">
+        <v>87000</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Surface Angle Mount</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>intercom-surface-angle-mount</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>5</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Junction Box</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Junction Box</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E98" t="n">
+        <v>66100</v>
+      </c>
+      <c r="F98" t="n">
+        <v>60100</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Junction Box</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>reader-pro-junction-box</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>5</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>UniFi G6 Entry</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>UniFi G6 Entry</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E99" t="n">
+        <v>557500</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>UniFi G6 Entry</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>g6-entry</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>5</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>UniFi G3 Elevator Starter Kit</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>UniFi G3 Elevator Starter Kit</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E100" t="n">
+        <v>2044700</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>UniFi G3 Elevator Starter Kit</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>g3-elevator-starter-kit</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>5</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>UniFi Access Button</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>UniFi Access Button</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E101" t="n">
+        <v>78300</v>
+      </c>
+      <c r="F101" t="n">
+        <v>71200</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>UniFi Access Button</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>access-button</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>5</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>UniFi Door Lock Relay Cable</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>UniFi Door Lock Relay Cable</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E102" t="n">
+        <v>237000</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>UniFi Door Lock Relay Cable</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>door-lock-relay-cable</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>5</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E103" t="n">
+        <v>448400</v>
+      </c>
+      <c r="F103" t="n">
+        <v>407700</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>UniFi Door Hub</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>door-hub</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>5</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>UniFi Enterprise Access Hub</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>UniFi Enterprise Access Hub</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E104" t="n">
+        <v>2203200</v>
+      </c>
+      <c r="F104" t="n">
+        <v>1858800</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>UniFi Enterprise Access Hub</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>enterprise-access-hub</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>5</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>UniFi Access Card (10-Pack)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>UniFi Access Card (10-Pack)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E105" t="n">
+        <v>61700</v>
+      </c>
+      <c r="F105" t="n">
+        <v>56100</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>UniFi Access Card</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>access-card-10pack</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>5</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>UniFi Pocket Keyfob, 10-Pack</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>UniFi Pocket Keyfob, 10-Pack</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E106" t="n">
+        <v>181800</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>UniFi Pocket Keyfob, 10-Pack</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>pocket-keyfob-10pack</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>5</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Wedge Mount</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Wedge Mount</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E107" t="n">
+        <v>99000</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Wedge Mount</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>intercom-wedge-mount</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>5</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Sunshield</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Sunshield</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E108" t="n">
+        <v>99000</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>UniFi Intercom Sunshield</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>intercom-sunshield</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>5</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Angle Mount</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Angle Mount</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E109" t="n">
+        <v>61800</v>
+      </c>
+      <c r="F109" t="n">
+        <v>56100</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro Angle Mount</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>reader-pro-angle-mount</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>5</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>UniFi Door Closer</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>UniFi Door Closer</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E110" t="n">
+        <v>259000</v>
+      </c>
+      <c r="F110" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>UniFi Door Closer</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>door-closer</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>5</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>UniFi PoE Over 2-Wire Retrofit Extender</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>UniFi PoE Over 2-Wire Retrofit Extender</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E111" t="n">
+        <v>194700</v>
+      </c>
+      <c r="F111" t="n">
+        <v>177000</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>UniFi PoE Over 2-Wire Retrofit Extender</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>poe-over-2wire-retrofit-extender</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>5</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E112" t="n">
+        <v>741800</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>UniFi Reader Pro</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>reader-pro</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>5</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit Hub</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit Hub</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E113" t="n">
+        <v>514500</v>
+      </c>
+      <c r="F113" t="n">
+        <v>467700</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit Hub</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>retrofit-hub</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>5</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>UniFi Reader Flex</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>UniFi Reader Flex</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E114" t="n">
+        <v>446400</v>
+      </c>
+      <c r="F114" t="n">
+        <v>405800</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>UniFi Reader Flex</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>reader-flex</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>5</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>UniFi Panic Bar</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>UniFi Panic Bar</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E115" t="n">
+        <v>873600</v>
+      </c>
+      <c r="F115" t="n">
+        <v>794200</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>UniFi Panic Bar</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>panic-bar</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>5</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>UniFi Access Ultra</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UniFi Access Ultra</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E116" t="n">
+        <v>251200</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>UniFi Access Ultra</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>access-ultra</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>5</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>UniFi Access Rescue KeySwitch</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UniFi Access Rescue KeySwitch</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E117" t="n">
+        <v>146500</v>
+      </c>
+      <c r="F117" t="n">
+        <v>133200</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>UniFi Access Rescue KeySwitch</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>access-rescue-keyswitch</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>5</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit PSU 12V</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit PSU 12V</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Door Access</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E118" t="n">
+        <v>150700</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>UniFi Retrofit PSU 12V</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>retrofit-psu-12v</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>5</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>U5G-Max</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>UniFi 5G Max</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E119" t="n">
+        <v>807300</v>
+      </c>
+      <c r="F119" t="n">
+        <v>807300</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>UniFi 5G Max</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>5g-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>UC-Cast-Lite</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>UniFi Display Cast Lite</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>UniFi Display Cast Lite</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>display-cast-lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>U-LTE-Backup Pro</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>UniFi LTE Backup Pro</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E121" t="n">
+        <v>527200</v>
+      </c>
+      <c r="F121" t="n">
+        <v>527200</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>UniFi LTE Backup Pro</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>lte-backup-pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>UMR</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E122" t="n">
+        <v>324300</v>
+      </c>
+      <c r="F122" t="n">
+        <v>324300</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>mobile-router</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>UMR-Industrial</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router Industrial</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router Industrial</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>mobile-router-industrial</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>UMR-Ultra</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router Ultra</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E124" t="n">
+        <v>228300</v>
+      </c>
+      <c r="F124" t="n">
+        <v>228300</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>UniFi Mobile Router Ultra</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>mobile-router-ultra</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>UPL-Port</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>UniFi PoE Audio Port</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E125" t="n">
+        <v>406600</v>
+      </c>
+      <c r="F125" t="n">
+        <v>406600</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>UniFi PoE Audio Port</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>poe-audio-port</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>UNAS-2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>UniFi UNAS 2</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E126" t="n">
+        <v>415600</v>
+      </c>
+      <c r="F126" t="n">
+        <v>415600</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>UniFi UNAS 2</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>unas-2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
미등록 4개 상품(WiFi BaseStation XG, G5 Dome Ultra, AirWire, G5 Pro) 상세페이지 제작 및 네이버 등록
NocoDB/대시보드 기준으로 판매 가능인데 상세페이지가 없어 등록되지 않은 상품 4개를
찾아 Ubiquiti 공식 스펙 조사 후 build_pages.py 패턴으로 상세페이지를 신규 제작하고
네이버 스마트스토어에 등록했다. Naver_Product_No를 TARGET_PRODUCTS에 추가해 NocoDB에
동기화하고(96개 → 100개), CLAUDE.md 현재 상태 섹션도 최신 수치로 정리하며 서술이
길어진 항목들을 HISTORY.md 참조로 축약했다.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/naver_상품등록_템플릿.xlsx
+++ b/naver_상품등록_템플릿.xlsx
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5378,6 +5378,170 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>UniFi WiFi BaseStation XG</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>유니파이 와이파이 베이스스테이션 XG</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>네트워크장비&gt;AP</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E127" t="n">
+        <v>3311000</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>UniFi WiFi BaseStation XG</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>wifi-basestation-xg</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>1</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>무료</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>UniFi G5 Dome Ultra</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>유니파이 UniFi G5 Dome Ultra</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>TV/영상가전&gt;CCTV</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>50002707</v>
+      </c>
+      <c r="E128" t="n">
+        <v>249000</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>UniFi G5 Dome Ultra</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>g5-dome-ultra</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>1</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>UniFi AirWire</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>유니파이 에어와이어</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>네트워크장비&gt;AP</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>50001623</v>
+      </c>
+      <c r="E129" t="n">
+        <v>444200</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>UniFi AirWire</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>airwire</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>1</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>무료</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>UniFi G5 Pro</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>유니파이 UniFi G5 Pro</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>TV/영상가전&gt;CCTV</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>50002707</v>
+      </c>
+      <c r="E130" t="n">
+        <v>836300</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>UniFi G5 Pro</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>g5-pro</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>1</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>